<commit_message>
i think it works pa check nlng
</commit_message>
<xml_diff>
--- a/output/item_analysis.xlsx
+++ b/output/item_analysis.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Item Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Student Results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Question Responses" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +466,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -500,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -509,9 +511,12 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -547,17 +552,32 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Number Correct</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Number Wrong</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Difficulty Index</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Discrimination Index</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Students Wrong</t>
         </is>
       </c>
     </row>
@@ -588,26 +608,37 @@
         </is>
       </c>
       <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>Review</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Maria Santos (wrong)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q014</t>
+          <t>Q003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Which symbol starts a Python comment?</t>
+          <t>Complete the code: print(______)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -617,23 +648,34 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MCQ</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>"Hello"</t>
         </is>
       </c>
       <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Review</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -664,26 +706,37 @@
         </is>
       </c>
       <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Review</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz (wrong)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q011</t>
+          <t>Q014</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Python keyword for a conditional branch is ______.</t>
+          <t>Which symbol starts a Python comment?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -693,61 +746,671 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FillBlank</t>
+          <t>MCQ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>if</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Review</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Maria Santos (wrong)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Q005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Which keyword defines a function?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MCQ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz (wrong)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Python Fundamentals</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Python Fundamentals</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Question ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Student Answer</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Answer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Is Correct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Student Score</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Student Percentage</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Q013</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Complete: name = "Ada"; print(______)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Q003</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Complete the code: print(______)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>"Hello"</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>"Hello"</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="n">
+        <v>60</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Q015</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The function used to find the length of a sequence is ______.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>len</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>60</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q014</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Which symbol starts a Python comment?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>60</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Q005</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Which keyword defines a function?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Juan Dela Cruz</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>60</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Q013</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Complete: name = "Ada"; print(______)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Q003</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Complete the code: print(______)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Python</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Programming</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>"Hello"</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>"Hello"</t>
+        </is>
+      </c>
+      <c r="F8" t="b">
         <v>1</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Q015</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The function used to find the length of a sequence is ______.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>len</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>len</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q014</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Which symbol starts a Python comment?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F10" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q005</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Which keyword defines a function?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-27T00:00:00+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>